<commit_message>
def setup inicial creeper
</commit_message>
<xml_diff>
--- a/python/creeper/planilla.xlsx
+++ b/python/creeper/planilla.xlsx
@@ -54,11 +54,4 @@
     </row>
   </sheetData>
 </worksheet>
-</file>
-
-<file path=creeper_infection/.creeper_marker.txt>CREEPER VIRUS - INFECTION MARKER
-Timestamp: 2026-07-08 17:47:49.804841
-Original file: planilla.xlsx
-This file was infected by the Creeper educational virus.
-
 </file>
</xml_diff>